<commit_message>
used a .py fix script to fix emojis coding in the backend
</commit_message>
<xml_diff>
--- a/comprehensive_grocery_certifications.xlsx
+++ b/comprehensive_grocery_certifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StardogChampion\TBL-Grocery-Scanner---DEVELOPMENT-VERSION-Active-development-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1CDC80-CD33-45AF-8D9E-43251CDF89FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DF5234-6FF9-4ADE-A23F-114E5B13D6ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31886,7 +31886,7 @@
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
         <f ca="1">NOW()</f>
-        <v>46099.813945486108</v>
+        <v>46099.985527199075</v>
       </c>
     </row>
   </sheetData>

</xml_diff>